<commit_message>
Finalised analysis for thesis
</commit_message>
<xml_diff>
--- a/Carbon/Cores.xlsx
+++ b/Carbon/Cores.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lukaseamus/Desktop/PhD/Papers/Burial/kelp-burial/Carbon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D437D40A-7F6E-D94C-A958-25BEB4F34263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A62427-AD5C-2748-A481-B2A2719459FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8040" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{D120C0EF-290F-244A-AE4B-CB2F7CD281C3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="107">
   <si>
     <t>ID</t>
   </si>
@@ -354,6 +354,9 @@
   </si>
   <si>
     <t>burrowing shrimp</t>
+  </si>
+  <si>
+    <t>crab (presumed dead)</t>
   </si>
 </sst>
 </file>
@@ -872,6 +875,9 @@
       <c r="H5" t="s">
         <v>50</v>
       </c>
+      <c r="I5" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">

</xml_diff>